<commit_message>
Outbound 2: vendorizar SheetJS 0.20.3 oficial (reemplaza npm:xlsx@0.18.5)
- vendor/xlsx.mjs sin modificar + LICENSE + VENDOR.md (origen y SHA-256)
- index.ts, tests y generacion de fixtures usan la libreria vendorizada
- 25/25 tests PASS; fixtures regenerados con 0.20.3; mismo resumen (11/4/1/6)

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01A8MAPh87mmi5ExZ5RmzhnY
</commit_message>
<xml_diff>
--- a/supabase/functions/prospect-import-preview/test/fixtures/trade_up_ficticio.xlsx
+++ b/supabase/functions/prospect-import-preview/test/fixtures/trade_up_ficticio.xlsx
@@ -857,7 +857,7 @@
       </c>
     </row>
     <row r="3">
-      <c r="A3">
+      <c r="A3" t="e">
         <f>2020+5</f>
       </c>
       <c r="B3" t="str">
@@ -866,7 +866,7 @@
       <c r="C3" t="str">
         <v/>
       </c>
-      <c r="D3">
+      <c r="D3" t="e">
         <f>2020+5</f>
       </c>
       <c r="E3" t="str">

</xml_diff>